<commit_message>
Complete Phase 3 functional test scenarios
</commit_message>
<xml_diff>
--- a/src/testData/LoginData.xlsx
+++ b/src/testData/LoginData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Study\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alfaj\eclipse-workspace\OpenCartHybridFramework\src\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{41471941-3B45-4A70-A919-794CE57E5B37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32523137-A7DB-484F-942F-19AB22F97748}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" xr2:uid="{0565196C-45AB-42EC-AD6B-AC66CC86E64E}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Usernames</t>
   </si>
@@ -60,28 +60,19 @@
     <t>Asawd@gmail.com</t>
   </si>
   <si>
-    <t>Supert@gmail.com</t>
-  </si>
-  <si>
-    <t>Mnxjbhjdb@gmail.com</t>
-  </si>
-  <si>
-    <t>Jones123@gmail.com</t>
-  </si>
-  <si>
-    <t>Jones123</t>
-  </si>
-  <si>
     <t>admin123</t>
   </si>
   <si>
     <t>hsbdygf</t>
   </si>
   <si>
-    <t>sjhbfhu</t>
-  </si>
-  <si>
-    <t>ihbfsddf</t>
+    <t>Expected Result</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valid </t>
+  </si>
+  <si>
+    <t>Invalid</t>
   </si>
 </sst>
 </file>
@@ -481,69 +472,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FF2ECA0-149E-48D7-9D6A-78EE47867381}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="19.19921875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>8</v>
+        <v>4</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A6" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>7</v>
+      <c r="C3" s="3" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{3FAF71BE-9C03-48F0-9FC3-212B48E0133A}"/>
-    <hyperlink ref="A4" r:id="rId2" xr:uid="{E3F1572F-6C6B-45DC-A4DA-6DA1603211B1}"/>
-    <hyperlink ref="A5" r:id="rId3" xr:uid="{E21B1B1C-E757-4A5C-9580-24BE34B603F0}"/>
-    <hyperlink ref="A6" r:id="rId4" xr:uid="{2AEEBEB3-7FF8-4D27-B21F-95D2EFA6A35E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>